<commit_message>
refine: focus text output on qualities, only mention standout/concern metrics
- Boring text now only includes metrics that are excellent/outstanding or
  below average/poor, not every notable one
- Prompt tells LLM to lead with qualities, reference metrics sparingly
- Few-shot examples updated to match new boring text format

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/gpt_examples/Physical.xlsx
+++ b/data/gpt_examples/Physical.xlsx
@@ -444,9 +444,9 @@
       <c r="A2" t="inlineStr">
         <is>
           <t>Here is a physical profile of Mohamed Salah Ghaly, who plays as a Wide Attacker for Liverpool Football Club in the ENG - Premier League. All ratings are compared against 187 Wide Attacker players.
-He was elite in Speed compared to other players in the same position group. He was above average in Acceleration compared to other players in the same position group. He was below average in Agility compared to other players in the same position group. He was well below average in Endurance compared to other players in the same position group.
-Notable strengths in underlying metrics: In PSV-99, which contributes to Speed, he was excellent. In TOP 5 PSV-99, which contributes to Speed, he was excellent. In TOP 3 Time to Sprint, which contributes to Acceleration, he was good. In TOP 3 Time to HSR post-COD, which contributes to Acceleration, he was good.
-Notable weaknesses in underlying metrics: In Change of Direction Count P90, which contributes to Agility, he was below average. In M/min P90, which contributes to Endurance, he was poor. In Distance P90, which contributes to Endurance, he was poor. In Running Distance P90, which contributes to Endurance, he was below average. In HSR Distance P90, which contributes to Endurance, he was below average.</t>
+He was elite in Speed compared to other players in the same position group. He was above average in Acceleration compared to other players in the same position group. He was below average in Agility compared to other players in the same position group. He was well below average in Endurance compared to other players in the same position group. 
+His PSV-99 (Speed) was excellent. His TOP 5 PSV-99 (Speed) was excellent.
+His Change of Direction Count P90 (Agility) was below average. His M/min P90 (Endurance) was poor. His Distance P90 (Endurance) was poor. His Running Distance P90 (Endurance) was below average. His HSR Distance P90 (Endurance) was below average.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -459,8 +459,8 @@
       <c r="A3" t="inlineStr">
         <is>
           <t>Here is a physical profile of Josko Gvardiol, who plays as a Central Defender for Manchester City in the ENG - Premier League. All ratings are compared against 524 Central Defender players.
-He was elite in Speed compared to other players in the same position group. He was exceptional in Acceleration compared to other players in the same position group. He was exceptional in Agility compared to other players in the same position group. He was elite in Endurance compared to other players in the same position group.
-Notable strengths in underlying metrics: In PSV-99, which contributes to Speed, he was excellent. In TOP 5 PSV-99, which contributes to Speed, he was excellent. In TOP 3 Time to Sprint, which contributes to Acceleration, he was outstanding. In TOP 3 Time to HSR, which contributes to Acceleration, he was excellent. In TOP 3 Time to Sprint post-COD, which contributes to Acceleration, he was excellent. In TOP 3 Time to HSR post-COD, which contributes to Acceleration, he was outstanding. In Explosive Acceleration to Sprint Count P90, which contributes to Acceleration, he was outstanding. In Explosive Acceleration to HSR Count P90, which contributes to Acceleration, he was outstanding. In Change of Direction Count P90, which contributes to Agility, he was outstanding. In M/min P90, which contributes to Endurance, he was good. In Distance P90, which contributes to Endurance, he was good. In Running Distance P90, which contributes to Endurance, he was excellent. In HSR Distance P90, which contributes to Endurance, he was outstanding.</t>
+He was elite in Speed compared to other players in the same position group. He was exceptional in Acceleration compared to other players in the same position group. He was exceptional in Agility compared to other players in the same position group. He was elite in Endurance compared to other players in the same position group. 
+His PSV-99 (Speed) was excellent. His TOP 5 PSV-99 (Speed) was excellent. His TOP 3 Time to Sprint (Acceleration) was outstanding. His TOP 3 Time to HSR (Acceleration) was excellent. His TOP 3 Time to Sprint post-COD (Acceleration) was excellent. His TOP 3 Time to HSR post-COD (Acceleration) was outstanding. His Explosive Acceleration to Sprint Count P90 (Acceleration) was outstanding. His Explosive Acceleration to HSR Count P90 (Acceleration) was outstanding. His Change of Direction Count P90 (Agility) was outstanding. His Running Distance P90 (Endurance) was excellent. His HSR Distance P90 (Endurance) was outstanding.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -472,10 +472,10 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Here is a physical profile of Rodrigo Hernandez Cascante, who plays as a Midfield for Manchester City in the ENG - Premier League. All ratings are compared against 451 Midfield players.
-He was below average in Speed compared to other players in the same position group. He was below average in Acceleration compared to other players in the same position group. He was below average in Agility compared to other players in the same position group. He was elite in Endurance compared to other players in the same position group.
-Notable strengths in underlying metrics: In M/min P90, which contributes to Endurance, he was excellent. In Distance P90, which contributes to Endurance, he was excellent. In Running Distance P90, which contributes to Endurance, he was outstanding.
-Notable weaknesses in underlying metrics: In TOP 5 PSV-99, which contributes to Speed, he was below average. In Explosive Acceleration to Sprint Count P90, which contributes to Acceleration, he was below average. In Explosive Acceleration to HSR Count P90, which contributes to Acceleration, he was poor.</t>
+          <t>Here is a physical profile of Rodrigo Hernández Cascante, who plays as a Midfield for Manchester City in the ENG - Premier League. All ratings are compared against 451 Midfield players.
+He was below average in Speed compared to other players in the same position group. He was below average in Acceleration compared to other players in the same position group. He was below average in Agility compared to other players in the same position group. He was elite in Endurance compared to other players in the same position group. 
+His M/min P90 (Endurance) was excellent. His Distance P90 (Endurance) was excellent. His Running Distance P90 (Endurance) was outstanding.
+His TOP 5 PSV-99 (Speed) was below average. His Explosive Acceleration to Sprint Count P90 (Acceleration) was below average. His Explosive Acceleration to HSR Count P90 (Acceleration) was poor.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -488,9 +488,9 @@
       <c r="A5" t="inlineStr">
         <is>
           <t>Here is a physical profile of Virgil van Dijk, who plays as a Central Defender for Liverpool Football Club in the ENG - Premier League. All ratings are compared against 524 Central Defender players.
-He was elite in Speed compared to other players in the same position group. He was elite in Acceleration compared to other players in the same position group. He was well below average in Agility compared to other players in the same position group. He was very poor in Endurance compared to other players in the same position group.
-Notable strengths in underlying metrics: In PSV-99, which contributes to Speed, he was good. In TOP 5 PSV-99, which contributes to Speed, he was outstanding. In TOP 3 Time to HSR, which contributes to Acceleration, he was excellent. In TOP 3 Time to HSR post-COD, which contributes to Acceleration, he was excellent. In Explosive Acceleration to Sprint Count P90, which contributes to Acceleration, he was excellent.
-Notable weaknesses in underlying metrics: In Change of Direction Count P90, which contributes to Agility, he was poor. In M/min P90, which contributes to Endurance, he was poor. In Distance P90, which contributes to Endurance, he was poor. In Running Distance P90, which contributes to Endurance, he was poor. In HSR Distance P90, which contributes to Endurance, he was poor.</t>
+He was elite in Speed compared to other players in the same position group. He was elite in Acceleration compared to other players in the same position group. He was well below average in Agility compared to other players in the same position group. He was very poor in Endurance compared to other players in the same position group. 
+His TOP 5 PSV-99 (Speed) was outstanding. His TOP 3 Time to HSR (Acceleration) was excellent. His TOP 3 Time to HSR post-COD (Acceleration) was excellent. His Explosive Acceleration to Sprint Count P90 (Acceleration) was excellent.
+His Change of Direction Count P90 (Agility) was poor. His M/min P90 (Endurance) was poor. His Distance P90 (Endurance) was poor. His Running Distance P90 (Endurance) was poor. His HSR Distance P90 (Endurance) was poor.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -503,9 +503,9 @@
       <c r="A6" t="inlineStr">
         <is>
           <t>Here is a physical profile of Harry Kane, who plays as a Center Forward for FC Bayern Munchen in the GER - Bundesliga. All ratings are compared against 278 Center Forward players.
-He was very poor in Speed compared to other players in the same position group. He was well below average in Acceleration compared to other players in the same position group. He was very poor in Agility compared to other players in the same position group. He was well above average in Endurance compared to other players in the same position group.
-Notable strengths in underlying metrics: In M/min P90, which contributes to Endurance, he was excellent. In Distance P90, which contributes to Endurance, he was excellent.
-Notable weaknesses in underlying metrics: In PSV-99, which contributes to Speed, he was poor. In TOP 5 PSV-99, which contributes to Speed, he was poor. In TOP 3 Time to Sprint, which contributes to Acceleration, he was poor. In TOP 3 Time to HSR, which contributes to Acceleration, he was poor. In TOP 3 Time to HSR post-COD, which contributes to Acceleration, he was below average. In Explosive Acceleration to Sprint Count P90, which contributes to Acceleration, he was poor. In Explosive Acceleration to HSR Count P90, which contributes to Acceleration, he was poor. In Change of Direction Count P90, which contributes to Agility, he was poor. In HSR Distance P90, which contributes to Endurance, he was poor.</t>
+He was very poor in Speed compared to other players in the same position group. He was well below average in Acceleration compared to other players in the same position group. He was very poor in Agility compared to other players in the same position group. He was well above average in Endurance compared to other players in the same position group. 
+His M/min P90 (Endurance) was excellent. His Distance P90 (Endurance) was excellent.
+His PSV-99 (Speed) was poor. His TOP 5 PSV-99 (Speed) was poor. His TOP 3 Time to Sprint (Acceleration) was poor. His TOP 3 Time to HSR (Acceleration) was poor. His TOP 3 Time to HSR post-COD (Acceleration) was below average. His Explosive Acceleration to Sprint Count P90 (Acceleration) was poor. His Explosive Acceleration to HSR Count P90 (Acceleration) was poor. His Change of Direction Count P90 (Agility) was poor. His HSR Distance P90 (Endurance) was poor.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">

</xml_diff>

<commit_message>
refine: use friendly metric names instead of raw column names
- PSV-99 → "top speed", TOP 5 PSV-99 → "average top speed", etc.
- All 15 underlying metrics now have readable names in the boring text
- Few-shot examples regenerated to match

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/gpt_examples/Physical.xlsx
+++ b/data/gpt_examples/Physical.xlsx
@@ -445,8 +445,8 @@
         <is>
           <t>Here is a physical profile of Mohamed Salah Ghaly, who plays as a Wide Attacker for Liverpool Football Club in the ENG - Premier League. All ratings are compared against 187 Wide Attacker players.
 He was elite in Speed compared to other players in the same position group. He was above average in Acceleration compared to other players in the same position group. He was below average in Agility compared to other players in the same position group. He was well below average in Endurance compared to other players in the same position group. 
-His PSV-99 (Speed) was excellent. His TOP 5 PSV-99 (Speed) was excellent.
-His Change of Direction Count P90 (Agility) was below average. His M/min P90 (Endurance) was poor. His Distance P90 (Endurance) was poor. His Running Distance P90 (Endurance) was below average. His HSR Distance P90 (Endurance) was below average.</t>
+His top speed (Speed) was excellent. His average top speed (Speed) was excellent.
+His change of direction frequency (Agility) was below average. His metres per minute (Endurance) was poor. His total distance covered (Endurance) was poor. His running distance (Endurance) was below average. His high-speed running distance (Endurance) was below average.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -460,7 +460,7 @@
         <is>
           <t>Here is a physical profile of Josko Gvardiol, who plays as a Central Defender for Manchester City in the ENG - Premier League. All ratings are compared against 524 Central Defender players.
 He was elite in Speed compared to other players in the same position group. He was exceptional in Acceleration compared to other players in the same position group. He was exceptional in Agility compared to other players in the same position group. He was elite in Endurance compared to other players in the same position group. 
-His PSV-99 (Speed) was excellent. His TOP 5 PSV-99 (Speed) was excellent. His TOP 3 Time to Sprint (Acceleration) was outstanding. His TOP 3 Time to HSR (Acceleration) was excellent. His TOP 3 Time to Sprint post-COD (Acceleration) was excellent. His TOP 3 Time to HSR post-COD (Acceleration) was outstanding. His Explosive Acceleration to Sprint Count P90 (Acceleration) was outstanding. His Explosive Acceleration to HSR Count P90 (Acceleration) was outstanding. His Change of Direction Count P90 (Agility) was outstanding. His Running Distance P90 (Endurance) was excellent. His HSR Distance P90 (Endurance) was outstanding.</t>
+His top speed (Speed) was excellent. His average top speed (Speed) was excellent. His time to reach sprint speed (Acceleration) was outstanding. His time to reach high-speed running (Acceleration) was excellent. His time to sprint after changing direction (Acceleration) was excellent. His time to reach high-speed running after changing direction (Acceleration) was outstanding. His explosive sprint burst volume (Acceleration) was outstanding. His explosive high-speed running burst volume (Acceleration) was outstanding. His change of direction frequency (Agility) was outstanding. His running distance (Endurance) was excellent. His high-speed running distance (Endurance) was outstanding.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -474,8 +474,8 @@
         <is>
           <t>Here is a physical profile of Rodrigo Hernández Cascante, who plays as a Midfield for Manchester City in the ENG - Premier League. All ratings are compared against 451 Midfield players.
 He was below average in Speed compared to other players in the same position group. He was below average in Acceleration compared to other players in the same position group. He was below average in Agility compared to other players in the same position group. He was elite in Endurance compared to other players in the same position group. 
-His M/min P90 (Endurance) was excellent. His Distance P90 (Endurance) was excellent. His Running Distance P90 (Endurance) was outstanding.
-His TOP 5 PSV-99 (Speed) was below average. His Explosive Acceleration to Sprint Count P90 (Acceleration) was below average. His Explosive Acceleration to HSR Count P90 (Acceleration) was poor.</t>
+His metres per minute (Endurance) was excellent. His total distance covered (Endurance) was excellent. His running distance (Endurance) was outstanding.
+His average top speed (Speed) was below average. His explosive sprint burst volume (Acceleration) was below average. His explosive high-speed running burst volume (Acceleration) was poor.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -489,8 +489,8 @@
         <is>
           <t>Here is a physical profile of Virgil van Dijk, who plays as a Central Defender for Liverpool Football Club in the ENG - Premier League. All ratings are compared against 524 Central Defender players.
 He was elite in Speed compared to other players in the same position group. He was elite in Acceleration compared to other players in the same position group. He was well below average in Agility compared to other players in the same position group. He was very poor in Endurance compared to other players in the same position group. 
-His TOP 5 PSV-99 (Speed) was outstanding. His TOP 3 Time to HSR (Acceleration) was excellent. His TOP 3 Time to HSR post-COD (Acceleration) was excellent. His Explosive Acceleration to Sprint Count P90 (Acceleration) was excellent.
-His Change of Direction Count P90 (Agility) was poor. His M/min P90 (Endurance) was poor. His Distance P90 (Endurance) was poor. His Running Distance P90 (Endurance) was poor. His HSR Distance P90 (Endurance) was poor.</t>
+His average top speed (Speed) was outstanding. His time to reach high-speed running (Acceleration) was excellent. His time to reach high-speed running after changing direction (Acceleration) was excellent. His explosive sprint burst volume (Acceleration) was excellent.
+His change of direction frequency (Agility) was poor. His metres per minute (Endurance) was poor. His total distance covered (Endurance) was poor. His running distance (Endurance) was poor. His high-speed running distance (Endurance) was poor.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -504,8 +504,8 @@
         <is>
           <t>Here is a physical profile of Harry Kane, who plays as a Center Forward for FC Bayern Munchen in the GER - Bundesliga. All ratings are compared against 278 Center Forward players.
 He was very poor in Speed compared to other players in the same position group. He was well below average in Acceleration compared to other players in the same position group. He was very poor in Agility compared to other players in the same position group. He was well above average in Endurance compared to other players in the same position group. 
-His M/min P90 (Endurance) was excellent. His Distance P90 (Endurance) was excellent.
-His PSV-99 (Speed) was poor. His TOP 5 PSV-99 (Speed) was poor. His TOP 3 Time to Sprint (Acceleration) was poor. His TOP 3 Time to HSR (Acceleration) was poor. His TOP 3 Time to HSR post-COD (Acceleration) was below average. His Explosive Acceleration to Sprint Count P90 (Acceleration) was poor. His Explosive Acceleration to HSR Count P90 (Acceleration) was poor. His Change of Direction Count P90 (Agility) was poor. His HSR Distance P90 (Endurance) was poor.</t>
+His metres per minute (Endurance) was excellent. His total distance covered (Endurance) was excellent.
+His top speed (Speed) was poor. His average top speed (Speed) was poor. His time to reach sprint speed (Acceleration) was poor. His time to reach high-speed running (Acceleration) was poor. His time to reach high-speed running after changing direction (Acceleration) was below average. His explosive sprint burst volume (Acceleration) was poor. His explosive high-speed running burst volume (Acceleration) was poor. His change of direction frequency (Agility) was poor. His high-speed running distance (Endurance) was poor.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">

</xml_diff>

<commit_message>
fix: remove attribute name in parentheses from metric callouts
'His top speed (Speed) was excellent' → 'His top speed was excellent'

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/gpt_examples/Physical.xlsx
+++ b/data/gpt_examples/Physical.xlsx
@@ -445,8 +445,8 @@
         <is>
           <t>Here is a physical profile of Mohamed Salah Ghaly, who plays as a Wide Attacker for Liverpool Football Club in the ENG - Premier League. All ratings are compared against 187 Wide Attacker players.
 He was elite in Speed compared to other players in the same position group. He was above average in Acceleration compared to other players in the same position group. He was below average in Agility compared to other players in the same position group. He was well below average in Endurance compared to other players in the same position group. 
-His top speed (Speed) was excellent. His average top speed (Speed) was excellent.
-His change of direction frequency (Agility) was below average. His metres per minute (Endurance) was poor. His total distance covered (Endurance) was poor. His running distance (Endurance) was below average. His high-speed running distance (Endurance) was below average.</t>
+His top speed was excellent. His average top speed was excellent.
+His change of direction frequency was below average. His metres per minute was poor. His total distance covered was poor. His running distance was below average. His high-speed running distance was below average.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -460,7 +460,7 @@
         <is>
           <t>Here is a physical profile of Josko Gvardiol, who plays as a Central Defender for Manchester City in the ENG - Premier League. All ratings are compared against 524 Central Defender players.
 He was elite in Speed compared to other players in the same position group. He was exceptional in Acceleration compared to other players in the same position group. He was exceptional in Agility compared to other players in the same position group. He was elite in Endurance compared to other players in the same position group. 
-His top speed (Speed) was excellent. His average top speed (Speed) was excellent. His time to reach sprint speed (Acceleration) was outstanding. His time to reach high-speed running (Acceleration) was excellent. His time to sprint after changing direction (Acceleration) was excellent. His time to reach high-speed running after changing direction (Acceleration) was outstanding. His explosive sprint burst volume (Acceleration) was outstanding. His explosive high-speed running burst volume (Acceleration) was outstanding. His change of direction frequency (Agility) was outstanding. His running distance (Endurance) was excellent. His high-speed running distance (Endurance) was outstanding.</t>
+His top speed was excellent. His average top speed was excellent. His time to reach sprint speed was outstanding. His time to reach high-speed running was excellent. His time to sprint after changing direction was excellent. His time to reach high-speed running after changing direction was outstanding. His explosive sprint burst volume was outstanding. His explosive high-speed running burst volume was outstanding. His change of direction frequency was outstanding. His running distance was excellent. His high-speed running distance was outstanding.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -474,8 +474,8 @@
         <is>
           <t>Here is a physical profile of Rodrigo Hernández Cascante, who plays as a Midfield for Manchester City in the ENG - Premier League. All ratings are compared against 451 Midfield players.
 He was below average in Speed compared to other players in the same position group. He was below average in Acceleration compared to other players in the same position group. He was below average in Agility compared to other players in the same position group. He was elite in Endurance compared to other players in the same position group. 
-His metres per minute (Endurance) was excellent. His total distance covered (Endurance) was excellent. His running distance (Endurance) was outstanding.
-His average top speed (Speed) was below average. His explosive sprint burst volume (Acceleration) was below average. His explosive high-speed running burst volume (Acceleration) was poor.</t>
+His metres per minute was excellent. His total distance covered was excellent. His running distance was outstanding.
+His average top speed was below average. His explosive sprint burst volume was below average. His explosive high-speed running burst volume was poor.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -489,8 +489,8 @@
         <is>
           <t>Here is a physical profile of Virgil van Dijk, who plays as a Central Defender for Liverpool Football Club in the ENG - Premier League. All ratings are compared against 524 Central Defender players.
 He was elite in Speed compared to other players in the same position group. He was elite in Acceleration compared to other players in the same position group. He was well below average in Agility compared to other players in the same position group. He was very poor in Endurance compared to other players in the same position group. 
-His average top speed (Speed) was outstanding. His time to reach high-speed running (Acceleration) was excellent. His time to reach high-speed running after changing direction (Acceleration) was excellent. His explosive sprint burst volume (Acceleration) was excellent.
-His change of direction frequency (Agility) was poor. His metres per minute (Endurance) was poor. His total distance covered (Endurance) was poor. His running distance (Endurance) was poor. His high-speed running distance (Endurance) was poor.</t>
+His average top speed was outstanding. His time to reach high-speed running was excellent. His time to reach high-speed running after changing direction was excellent. His explosive sprint burst volume was excellent.
+His change of direction frequency was poor. His metres per minute was poor. His total distance covered was poor. His running distance was poor. His high-speed running distance was poor.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -504,8 +504,8 @@
         <is>
           <t>Here is a physical profile of Harry Kane, who plays as a Center Forward for FC Bayern Munchen in the GER - Bundesliga. All ratings are compared against 278 Center Forward players.
 He was very poor in Speed compared to other players in the same position group. He was well below average in Acceleration compared to other players in the same position group. He was very poor in Agility compared to other players in the same position group. He was well above average in Endurance compared to other players in the same position group. 
-His metres per minute (Endurance) was excellent. His total distance covered (Endurance) was excellent.
-His top speed (Speed) was poor. His average top speed (Speed) was poor. His time to reach sprint speed (Acceleration) was poor. His time to reach high-speed running (Acceleration) was poor. His time to reach high-speed running after changing direction (Acceleration) was below average. His explosive sprint burst volume (Acceleration) was poor. His explosive high-speed running burst volume (Acceleration) was poor. His change of direction frequency (Agility) was poor. His high-speed running distance (Endurance) was poor.</t>
+His metres per minute was excellent. His total distance covered was excellent.
+His top speed was poor. His average top speed was poor. His time to reach sprint speed was poor. His time to reach high-speed running was poor. His time to reach high-speed running after changing direction was below average. His explosive sprint burst volume was poor. His explosive high-speed running burst volume was poor. His change of direction frequency was poor. His high-speed running distance was poor.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">

</xml_diff>

<commit_message>
fix: use z-score thresholds for word labels instead of percentiles
The course framework uses z-scores (outstanding/excellent/good/average/
below average/poor) not percentile buckets. Now computes z-scores within
position group from the attribute scores and applies the standard
thresholds. Few-shot examples updated to match.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/gpt_examples/Physical.xlsx
+++ b/data/gpt_examples/Physical.xlsx
@@ -1,37 +1,95 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+  <si>
+    <t>user</t>
+  </si>
+  <si>
+    <t>assistant</t>
+  </si>
+  <si>
+    <t>Here is a physical profile of Mohamed Salah Ghaly, who plays as a Wide Attacker for Liverpool Football Club in the ENG - Premier League. All ratings are compared against 187 Wide Attacker players.
+He was excellent in Speed compared to other players in the same position group. He was average in Acceleration compared to other players in the same position group. He was poor in Agility compared to other players in the same position group. He was poor in Endurance compared to other players in the same position group. 
+His top speed was excellent. His average top speed was excellent.
+His change of direction frequency was below average. His metres per minute was poor. His total distance covered was poor. His running distance was below average. His high-speed running distance was below average.</t>
+  </si>
+  <si>
+    <t>Here is a physical profile of Josko Gvardiol, who plays as a Central Defender for Manchester City in the ENG - Premier League. All ratings are compared against 524 Central Defender players.
+He was excellent in Speed compared to other players in the same position group. He was outstanding in Acceleration compared to other players in the same position group. He was outstanding in Agility compared to other players in the same position group. He was excellent in Endurance compared to other players in the same position group. 
+His top speed was excellent. His average top speed was excellent. His time to reach sprint speed was outstanding. His time to reach high-speed running was excellent. His time to sprint after changing direction was excellent. His time to reach high-speed running after changing direction was outstanding. His explosive sprint burst volume was outstanding. His explosive high-speed running burst volume was outstanding. His change of direction frequency was outstanding. His running distance was excellent. His high-speed running distance was outstanding.</t>
+  </si>
+  <si>
+    <t>Here is a physical profile of Rodrigo Hernández Cascante, who plays as a Midfield for Manchester City in the ENG - Premier League. All ratings are compared against 451 Midfield players.
+He was below average in Speed compared to other players in the same position group. He was below average in Acceleration compared to other players in the same position group. He was average in Agility compared to other players in the same position group. He was excellent in Endurance compared to other players in the same position group. 
+His metres per minute was excellent. His total distance covered was excellent. His running distance was outstanding.
+His average top speed was below average. His explosive sprint burst volume was below average. His explosive high-speed running burst volume was poor.</t>
+  </si>
+  <si>
+    <t>Here is a physical profile of Virgil van Dijk, who plays as a Central Defender for Liverpool Football Club in the ENG - Premier League. All ratings are compared against 524 Central Defender players.
+He was excellent in Speed compared to other players in the same position group. He was outstanding in Acceleration compared to other players in the same position group. He was poor in Agility compared to other players in the same position group. He was poor in Endurance compared to other players in the same position group. 
+His average top speed was outstanding. His time to reach high-speed running was excellent. His time to reach high-speed running after changing direction was excellent. His explosive sprint burst volume was excellent.
+His change of direction frequency was poor. His metres per minute was poor. His total distance covered was poor. His running distance was poor. His high-speed running distance was poor.</t>
+  </si>
+  <si>
+    <t>Here is a physical profile of Harry Kane, who plays as a Center Forward for FC Bayern Munchen in the GER - Bundesliga. All ratings are compared against 278 Center Forward players.
+He was poor in Speed compared to other players in the same position group. He was poor in Acceleration compared to other players in the same position group. He was poor in Agility compared to other players in the same position group. He was good in Endurance compared to other players in the same position group. 
+His metres per minute was excellent. His total distance covered was excellent.
+His top speed was poor. His average top speed was poor. His time to reach sprint speed was poor. His time to reach high-speed running was poor. His time to reach high-speed running after changing direction was below average. His explosive sprint burst volume was poor. His explosive high-speed running burst volume was poor. His change of direction frequency was poor. His high-speed running distance was poor.</t>
+  </si>
+  <si>
+    <t>In the Premier League this season, Mohamed Salah has showcased excellent speed, consistently ranking among the quickest wide attackers. His acceleration is average for the position, though he shows good ability to reach sprint speed and recover pace after changes of direction. His agility and endurance are both poor for a wide attacker, with low distance output and limited change of direction frequency. This is a player whose physical profile is built around short, explosive speed — devastating in those moments, but not one to press relentlessly or sustain high output across the full match.</t>
+  </si>
+  <si>
+    <t>Gvardiol has been a standout physical performer for Manchester City this season, with outstanding acceleration and agility combined with excellent speed and endurance. Every single underlying metric across all four attributes is notably strong — that is extremely rare for any player, let alone a central defender. His explosive burst volume and change of direction frequency are outstanding, and he sustains that intensity with excellent running distance and high-speed running output. This is a physically complete central defender with the ability to dominate in any tactical system.</t>
+  </si>
+  <si>
+    <t>In the Premier League this season, Rodri has showcased excellent endurance capabilities among midfielders, with outstanding running distance and excellent total distance covered and metres per minute. His speed and acceleration are both below average, and his agility is average for the position. His physical profile is centred entirely around sustained effort rather than explosive actions, making him a player whose contributions are built on covering ground consistently rather than making sharp, high-speed interventions.</t>
+  </si>
+  <si>
+    <t>Van Dijk has been a physically impressive performer for Liverpool this season, with excellent speed and outstanding acceleration among central defenders. His top speed and explosive sprint burst volume are both excellent, and his ability to reach high-speed running after changing direction is outstanding. His agility and endurance are both poor — he rarely changes direction compared to other centre-backs and his distance output is among the lowest in the position group. This is a defender whose physical value is entirely in his pace and explosiveness, ideally suited to a high defensive line where recovery speed matters most.</t>
+  </si>
+  <si>
+    <t>Kane has shown good endurance qualities for Bayern Munich this season, with excellent total distance covered and metres per minute output among centre forwards. His speed, acceleration, and agility are all poor for the position, with low top speed, slow acceleration times, and minimal change of direction activity. His high-speed running distance is also poor despite the strong overall distance output, suggesting his movement is deliberate and positional rather than explosive. This is a player whose contributions are built around consistent effort and intelligent positioning rather than any physical advantage.</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
   <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,93 +104,35 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -420,101 +420,59 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>user</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>assistant</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Here is a physical profile of Mohamed Salah Ghaly, who plays as a Wide Attacker for Liverpool Football Club in the ENG - Premier League. All ratings are compared against 187 Wide Attacker players.
-He was elite in Speed compared to other players in the same position group. He was above average in Acceleration compared to other players in the same position group. He was below average in Agility compared to other players in the same position group. He was well below average in Endurance compared to other players in the same position group. 
-His top speed was excellent. His average top speed was excellent.
-His change of direction frequency was below average. His metres per minute was poor. His total distance covered was poor. His running distance was below average. His high-speed running distance was below average.</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>In the Premier League this season, Mohamed Salah has showcased his elite speed, consistently ranking among the top wide attackers. His above average acceleration adds a valuable dimension to his attacking play, particularly in reaching sprint speed and recovering pace after changes of direction. While he maintains below average agility and struggles with endurance metrics, his outstanding speed capabilities highlight his potential as an explosive wide attacker who excels in decisive moments.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Here is a physical profile of Josko Gvardiol, who plays as a Central Defender for Manchester City in the ENG - Premier League. All ratings are compared against 524 Central Defender players.
-He was elite in Speed compared to other players in the same position group. He was exceptional in Acceleration compared to other players in the same position group. He was exceptional in Agility compared to other players in the same position group. He was elite in Endurance compared to other players in the same position group. 
-His top speed was excellent. His average top speed was excellent. His time to reach sprint speed was outstanding. His time to reach high-speed running was excellent. His time to sprint after changing direction was excellent. His time to reach high-speed running after changing direction was outstanding. His explosive sprint burst volume was outstanding. His explosive high-speed running burst volume was outstanding. His change of direction frequency was outstanding. His running distance was excellent. His high-speed running distance was outstanding.</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Gvardiol has been a standout physical performer for Manchester City this season, showcasing exceptional capabilities across all four key attributes. He excels in both speed and endurance at an elite level, while also demonstrating exceptional acceleration and agility. His outstanding explosive burst volume and change of direction frequency add a valuable dimension to his defensive play. Overall, he's performed at an outstanding level, demonstrating the qualities of a physically complete central defender with the rare ability to sustain high-intensity output across the full match.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Here is a physical profile of Rodrigo Hernández Cascante, who plays as a Midfield for Manchester City in the ENG - Premier League. All ratings are compared against 451 Midfield players.
-He was below average in Speed compared to other players in the same position group. He was below average in Acceleration compared to other players in the same position group. He was below average in Agility compared to other players in the same position group. He was elite in Endurance compared to other players in the same position group. 
-His metres per minute was excellent. His total distance covered was excellent. His running distance was outstanding.
-His average top speed was below average. His explosive sprint burst volume was below average. His explosive high-speed running burst volume was poor.</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>In the Premier League this season, Rodri has showcased his elite endurance capabilities, consistently ranking among the top midfielders in distance covered and metres per minute. His outstanding running distance highlights his sustained physical output across matches. While he maintains below average performance levels in speed, acceleration, and agility, his exceptional endurance contributions are notable, making him a player whose physical profile is centred around sustained effort rather than explosive actions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Here is a physical profile of Virgil van Dijk, who plays as a Central Defender for Liverpool Football Club in the ENG - Premier League. All ratings are compared against 524 Central Defender players.
-He was elite in Speed compared to other players in the same position group. He was elite in Acceleration compared to other players in the same position group. He was well below average in Agility compared to other players in the same position group. He was very poor in Endurance compared to other players in the same position group. 
-His average top speed was outstanding. His time to reach high-speed running was excellent. His time to reach high-speed running after changing direction was excellent. His explosive sprint burst volume was excellent.
-His change of direction frequency was poor. His metres per minute was poor. His total distance covered was poor. His running distance was poor. His high-speed running distance was poor.</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Van Dijk has been a physically impressive performer for Liverpool this season, showcasing elite speed and acceleration capabilities among central defenders. His outstanding top speed and excellent ability to reach high-speed running, including after changes of direction, add a valuable dimension to his defensive play. While he maintains well below average agility and struggles with endurance metrics across distance, running output, and metres per minute, his exceptional speed and explosive acceleration highlight his qualities as a physically dominant central defender.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Here is a physical profile of Harry Kane, who plays as a Center Forward for FC Bayern Munchen in the GER - Bundesliga. All ratings are compared against 278 Center Forward players.
-He was very poor in Speed compared to other players in the same position group. He was well below average in Acceleration compared to other players in the same position group. He was very poor in Agility compared to other players in the same position group. He was well above average in Endurance compared to other players in the same position group. 
-His metres per minute was excellent. His total distance covered was excellent.
-His top speed was poor. His average top speed was poor. His time to reach sprint speed was poor. His time to reach high-speed running was poor. His time to reach high-speed running after changing direction was below average. His explosive sprint burst volume was poor. His explosive high-speed running burst volume was poor. His change of direction frequency was poor. His high-speed running distance was poor.</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Kane has shown notable endurance qualities for Bayern Munich this season, showcasing excellent distance covered and metres per minute output among centre forwards. While he struggles with speed, acceleration, and agility metrics, maintaining very poor and well below average performance levels respectively, his sustained physical output highlights his capacity to contribute across the full match. His overall physical profile suggests a player whose contributions are built around consistent effort rather than explosive actions.</t>
-        </is>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>